<commit_message>
Update INARA 2026-09-07 11:48:57
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -795,7 +795,7 @@
         <v>1</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
@@ -839,7 +839,7 @@
         <v>0</v>
       </c>
       <c r="M3">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
@@ -2334,7 +2334,7 @@
         <v>1</v>
       </c>
       <c r="M35">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N35" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-08 14:35:34
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="115">
   <si>
     <t>ODP</t>
   </si>
@@ -49,13 +49,19 @@
     <t>OCCUPANCY_TERBARU</t>
   </si>
   <si>
-    <t>TOTAL_PS_USED</t>
-  </si>
-  <si>
-    <t>JUMLAH_VISIT_FM_MTD</t>
-  </si>
-  <si>
-    <t>VISITED</t>
+    <t>USED_ODP_IHLD_TERBARU</t>
+  </si>
+  <si>
+    <t>PS_BASELINE</t>
+  </si>
+  <si>
+    <t>PS_DIAKUI</t>
+  </si>
+  <si>
+    <t>JUMLAH_VISIT_MTD</t>
+  </si>
+  <si>
+    <t>VISITED_MTD</t>
   </si>
   <si>
     <t>MATCH_ODP_IHLD</t>
@@ -710,10 +716,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O43"/>
+  <dimension ref="A1:Q43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -759,28 +765,34 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:15">
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -789,42 +801,48 @@
         <v>0</v>
       </c>
       <c r="K2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2">
-        <v>5</v>
-      </c>
-      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+      <c r="N2">
         <v>1</v>
       </c>
-      <c r="O2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15">
+      <c r="O2">
+        <v>4</v>
+      </c>
+      <c r="P2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I3">
         <v>-8.526441949000001</v>
@@ -833,45 +851,51 @@
         <v>115.1364796</v>
       </c>
       <c r="K3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L3">
         <v>0</v>
       </c>
       <c r="M3">
-        <v>24</v>
-      </c>
-      <c r="N3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>6</v>
+      </c>
+      <c r="P3" t="b">
         <v>1</v>
       </c>
-      <c r="O3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15">
+      <c r="Q3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -880,45 +904,51 @@
         <v>0</v>
       </c>
       <c r="K4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
         <v>1</v>
       </c>
-      <c r="N4" t="b">
-        <v>1</v>
-      </c>
-      <c r="O4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15">
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I5">
         <v>-8.602367258999999</v>
@@ -927,45 +957,51 @@
         <v>116.1430562</v>
       </c>
       <c r="K5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
       <c r="M5">
-        <v>4</v>
-      </c>
-      <c r="N5" t="b">
-        <v>1</v>
-      </c>
-      <c r="O5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I6">
         <v>-8.603221198</v>
@@ -974,45 +1010,51 @@
         <v>116.143717</v>
       </c>
       <c r="K6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6">
-        <v>8</v>
-      </c>
-      <c r="N6" t="b">
-        <v>1</v>
-      </c>
-      <c r="O6" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I7">
         <v>-8.599239378</v>
@@ -1021,45 +1063,51 @@
         <v>116.1329936</v>
       </c>
       <c r="K7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7">
-        <v>3</v>
-      </c>
-      <c r="N7" t="b">
-        <v>1</v>
-      </c>
-      <c r="O7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I8">
         <v>-8.627093541000001</v>
@@ -1068,45 +1116,51 @@
         <v>116.1328874</v>
       </c>
       <c r="K8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8">
-        <v>1</v>
-      </c>
-      <c r="N8" t="b">
-        <v>1</v>
-      </c>
-      <c r="O8" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -1115,45 +1169,51 @@
         <v>0</v>
       </c>
       <c r="K9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L9">
         <v>0</v>
       </c>
       <c r="M9">
-        <v>1</v>
-      </c>
-      <c r="N9" t="b">
-        <v>1</v>
-      </c>
-      <c r="O9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I10">
         <v>-8.358494758999999</v>
@@ -1162,45 +1222,51 @@
         <v>116.1495849</v>
       </c>
       <c r="K10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10">
-        <v>1</v>
-      </c>
-      <c r="N10" t="b">
-        <v>1</v>
-      </c>
-      <c r="O10" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -1209,45 +1275,51 @@
         <v>0</v>
       </c>
       <c r="K11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L11">
         <v>0</v>
       </c>
       <c r="M11">
-        <v>1</v>
-      </c>
-      <c r="N11" t="b">
-        <v>1</v>
-      </c>
-      <c r="O11" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E12" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H12" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I12">
         <v>-8.34948075</v>
@@ -1256,45 +1328,51 @@
         <v>116.1686008</v>
       </c>
       <c r="K12" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L12">
         <v>0</v>
       </c>
       <c r="M12">
-        <v>1</v>
-      </c>
-      <c r="N12" t="b">
-        <v>1</v>
-      </c>
-      <c r="O12" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H13" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I13">
         <v>-8.347617261</v>
@@ -1303,45 +1381,51 @@
         <v>116.1690833</v>
       </c>
       <c r="K13" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
       <c r="M13">
-        <v>1</v>
-      </c>
-      <c r="N13" t="b">
-        <v>1</v>
-      </c>
-      <c r="O13" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C14" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D14" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E14" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F14" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G14" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H14" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I14">
         <v>-8.587127515000001</v>
@@ -1350,45 +1434,51 @@
         <v>116.3125604</v>
       </c>
       <c r="K14" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L14">
         <v>0</v>
       </c>
       <c r="M14">
-        <v>1</v>
-      </c>
-      <c r="N14" t="b">
-        <v>1</v>
-      </c>
-      <c r="O14" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C15" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E15" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G15" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H15" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I15">
         <v>-8.586417143</v>
@@ -1397,45 +1487,51 @@
         <v>116.3120566</v>
       </c>
       <c r="K15" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L15">
         <v>0</v>
       </c>
       <c r="M15">
-        <v>1</v>
-      </c>
-      <c r="N15" t="b">
-        <v>1</v>
-      </c>
-      <c r="O15" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F16" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G16" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H16" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I16">
         <v>-8.586269807000001</v>
@@ -1444,45 +1540,51 @@
         <v>116.3106078</v>
       </c>
       <c r="K16" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L16">
         <v>0</v>
       </c>
       <c r="M16">
-        <v>1</v>
-      </c>
-      <c r="N16" t="b">
-        <v>1</v>
-      </c>
-      <c r="O16" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B17" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G17" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H17" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I17">
         <v>-8.586482159999999</v>
@@ -1491,45 +1593,51 @@
         <v>116.3092842</v>
       </c>
       <c r="K17" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L17">
         <v>0</v>
       </c>
       <c r="M17">
-        <v>1</v>
-      </c>
-      <c r="N17" t="b">
-        <v>1</v>
-      </c>
-      <c r="O17" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B18" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C18" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E18" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F18" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G18" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H18" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I18">
         <v>-8.587142588000001</v>
@@ -1538,45 +1646,51 @@
         <v>116.3086122</v>
       </c>
       <c r="K18" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L18">
         <v>0</v>
       </c>
       <c r="M18">
-        <v>1</v>
-      </c>
-      <c r="N18" t="b">
-        <v>1</v>
-      </c>
-      <c r="O18" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B19" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C19" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F19" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G19" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H19" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I19">
         <v>-8.587113602000001</v>
@@ -1585,45 +1699,51 @@
         <v>116.3080444</v>
       </c>
       <c r="K19" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L19">
         <v>0</v>
       </c>
       <c r="M19">
-        <v>1</v>
-      </c>
-      <c r="N19" t="b">
-        <v>1</v>
-      </c>
-      <c r="O19" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17">
       <c r="A20" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B20" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C20" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D20" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E20" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G20" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H20" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I20">
         <v>-8.587634986999999</v>
@@ -1632,45 +1752,51 @@
         <v>116.307917</v>
       </c>
       <c r="K20" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L20">
         <v>0</v>
       </c>
       <c r="M20">
-        <v>1</v>
-      </c>
-      <c r="N20" t="b">
-        <v>1</v>
-      </c>
-      <c r="O20" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17">
       <c r="A21" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B21" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C21" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D21" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H21" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I21">
         <v>-8.589391066999999</v>
@@ -1679,45 +1805,51 @@
         <v>116.3103036</v>
       </c>
       <c r="K21" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L21">
         <v>0</v>
       </c>
       <c r="M21">
-        <v>1</v>
-      </c>
-      <c r="N21" t="b">
-        <v>1</v>
-      </c>
-      <c r="O21" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N21">
+        <v>0</v>
+      </c>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B22" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C22" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D22" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E22" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F22" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G22" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H22" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I22">
         <v>-8.589132962000001</v>
@@ -1726,45 +1858,51 @@
         <v>116.3069518</v>
       </c>
       <c r="K22" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L22">
         <v>0</v>
       </c>
       <c r="M22">
-        <v>1</v>
-      </c>
-      <c r="N22" t="b">
-        <v>1</v>
-      </c>
-      <c r="O22" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N22">
+        <v>0</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17">
       <c r="A23" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B23" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E23" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F23" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H23" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I23">
         <v>-8.589625893999999</v>
@@ -1773,45 +1911,51 @@
         <v>116.3057965</v>
       </c>
       <c r="K23" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L23">
         <v>0</v>
       </c>
       <c r="M23">
-        <v>1</v>
-      </c>
-      <c r="N23" t="b">
-        <v>1</v>
-      </c>
-      <c r="O23" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N23">
+        <v>0</v>
+      </c>
+      <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="P23" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C24" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D24" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E24" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F24" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G24" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H24" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I24">
         <v>-8.588048634</v>
@@ -1820,45 +1964,51 @@
         <v>116.3472497</v>
       </c>
       <c r="K24" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L24">
         <v>0</v>
       </c>
       <c r="M24">
-        <v>1</v>
-      </c>
-      <c r="N24" t="b">
-        <v>1</v>
-      </c>
-      <c r="O24" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17">
       <c r="A25" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C25" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D25" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E25" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G25" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H25" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I25">
         <v>0</v>
@@ -1867,45 +2017,51 @@
         <v>0</v>
       </c>
       <c r="K25" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="L25">
         <v>4</v>
       </c>
       <c r="M25">
-        <v>1</v>
-      </c>
-      <c r="N25" t="b">
-        <v>1</v>
-      </c>
-      <c r="O25" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15">
+        <v>4</v>
+      </c>
+      <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17">
       <c r="A26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B26" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C26" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D26" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E26" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G26" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H26" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I26">
         <v>-8.589379918000001</v>
@@ -1914,45 +2070,51 @@
         <v>116.3183431</v>
       </c>
       <c r="K26" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L26">
         <v>0</v>
       </c>
       <c r="M26">
-        <v>1</v>
-      </c>
-      <c r="N26" t="b">
-        <v>1</v>
-      </c>
-      <c r="O26" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N26">
+        <v>0</v>
+      </c>
+      <c r="O26">
+        <v>0</v>
+      </c>
+      <c r="P26" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B27" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C27" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E27" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F27" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G27" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H27" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I27">
         <v>-8.589138937</v>
@@ -1961,45 +2123,51 @@
         <v>116.307804</v>
       </c>
       <c r="K27" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L27">
         <v>0</v>
       </c>
       <c r="M27">
-        <v>1</v>
-      </c>
-      <c r="N27" t="b">
-        <v>1</v>
-      </c>
-      <c r="O27" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>0</v>
+      </c>
+      <c r="P27" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17">
       <c r="A28" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B28" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C28" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D28" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E28" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F28" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G28" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H28" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I28">
         <v>0</v>
@@ -2008,45 +2176,51 @@
         <v>0</v>
       </c>
       <c r="K28" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L28">
         <v>1</v>
       </c>
       <c r="M28">
+        <v>0</v>
+      </c>
+      <c r="N28">
         <v>1</v>
       </c>
-      <c r="N28" t="b">
-        <v>1</v>
-      </c>
-      <c r="O28" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15">
+      <c r="O28">
+        <v>0</v>
+      </c>
+      <c r="P28" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B29" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C29" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D29" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E29" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F29" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G29" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H29" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I29">
         <v>-8.592359</v>
@@ -2055,45 +2229,51 @@
         <v>116.2898168</v>
       </c>
       <c r="K29" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L29">
         <v>0</v>
       </c>
       <c r="M29">
-        <v>1</v>
-      </c>
-      <c r="N29" t="b">
-        <v>1</v>
-      </c>
-      <c r="O29" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29">
+        <v>0</v>
+      </c>
+      <c r="P29" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17">
       <c r="A30" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B30" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C30" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D30" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E30" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F30" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G30" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H30" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I30">
         <v>-8.616699897</v>
@@ -2102,45 +2282,51 @@
         <v>116.3165238</v>
       </c>
       <c r="K30" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L30">
         <v>0</v>
       </c>
       <c r="M30">
-        <v>1</v>
-      </c>
-      <c r="N30" t="b">
-        <v>1</v>
-      </c>
-      <c r="O30" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N30">
+        <v>0</v>
+      </c>
+      <c r="O30">
+        <v>0</v>
+      </c>
+      <c r="P30" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17">
       <c r="A31" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B31" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C31" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D31" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E31" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F31" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G31" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H31" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I31">
         <v>0</v>
@@ -2149,45 +2335,51 @@
         <v>0</v>
       </c>
       <c r="K31" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L31">
         <v>0</v>
       </c>
       <c r="M31">
-        <v>1</v>
-      </c>
-      <c r="N31" t="b">
-        <v>1</v>
-      </c>
-      <c r="O31" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N31">
+        <v>0</v>
+      </c>
+      <c r="O31">
+        <v>0</v>
+      </c>
+      <c r="P31" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17">
       <c r="A32" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B32" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C32" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D32" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E32" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F32" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G32" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H32" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I32">
         <v>-8.707284808000001</v>
@@ -2196,42 +2388,48 @@
         <v>116.2666262</v>
       </c>
       <c r="K32" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L32">
         <v>0</v>
       </c>
       <c r="M32">
-        <v>2</v>
-      </c>
-      <c r="N32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N32">
+        <v>0</v>
+      </c>
+      <c r="O32">
         <v>1</v>
       </c>
-      <c r="O32" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15">
+      <c r="P32" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17">
       <c r="A33" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B33" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C33" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D33" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F33" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G33" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H33" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I33">
         <v>0</v>
@@ -2240,42 +2438,48 @@
         <v>0</v>
       </c>
       <c r="K33" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="L33">
         <v>2</v>
       </c>
       <c r="M33">
-        <v>5</v>
-      </c>
-      <c r="N33" t="b">
-        <v>1</v>
-      </c>
-      <c r="O33" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15">
+        <v>2</v>
+      </c>
+      <c r="N33">
+        <v>0</v>
+      </c>
+      <c r="O33">
+        <v>0</v>
+      </c>
+      <c r="P33" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17">
       <c r="A34" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B34" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C34" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D34" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F34" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G34" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H34" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I34">
         <v>-10.15797653</v>
@@ -2284,42 +2488,48 @@
         <v>123.6662125</v>
       </c>
       <c r="K34" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L34">
         <v>0</v>
       </c>
       <c r="M34">
-        <v>5</v>
-      </c>
-      <c r="N34" t="b">
-        <v>1</v>
-      </c>
-      <c r="O34" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N34">
+        <v>0</v>
+      </c>
+      <c r="O34">
+        <v>0</v>
+      </c>
+      <c r="P34" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17">
       <c r="A35" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B35" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C35" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D35" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F35" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G35" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H35" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I35">
         <v>0</v>
@@ -2328,42 +2538,48 @@
         <v>0</v>
       </c>
       <c r="K35" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L35">
         <v>1</v>
       </c>
       <c r="M35">
-        <v>9</v>
-      </c>
-      <c r="N35" t="b">
+        <v>0</v>
+      </c>
+      <c r="N35">
         <v>1</v>
       </c>
-      <c r="O35" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15">
+      <c r="O35">
+        <v>1</v>
+      </c>
+      <c r="P35" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17">
       <c r="A36" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B36" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C36" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D36" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F36" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G36" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H36" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I36">
         <v>0</v>
@@ -2372,42 +2588,48 @@
         <v>0</v>
       </c>
       <c r="K36" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="L36">
         <v>2</v>
       </c>
       <c r="M36">
-        <v>3</v>
-      </c>
-      <c r="N36" t="b">
         <v>1</v>
       </c>
-      <c r="O36" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15">
+      <c r="N36">
+        <v>1</v>
+      </c>
+      <c r="O36">
+        <v>0</v>
+      </c>
+      <c r="P36" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17">
       <c r="A37" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B37" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C37" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D37" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F37" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G37" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H37" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I37">
         <v>-8.36708297</v>
@@ -2416,42 +2638,48 @@
         <v>115.1921949</v>
       </c>
       <c r="K37" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L37">
         <v>0</v>
       </c>
       <c r="M37">
-        <v>9</v>
-      </c>
-      <c r="N37" t="b">
-        <v>1</v>
-      </c>
-      <c r="O37" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15">
+        <v>0</v>
+      </c>
+      <c r="N37">
+        <v>0</v>
+      </c>
+      <c r="O37">
+        <v>0</v>
+      </c>
+      <c r="P37" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17">
       <c r="A38" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B38" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C38" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D38" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F38" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G38" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H38" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I38">
         <v>-8.364740604</v>
@@ -2460,42 +2688,48 @@
         <v>115.1918556</v>
       </c>
       <c r="K38" t="s">
+        <v>112</v>
+      </c>
+      <c r="L38">
+        <v>0</v>
+      </c>
+      <c r="M38">
+        <v>0</v>
+      </c>
+      <c r="N38">
+        <v>0</v>
+      </c>
+      <c r="O38">
+        <v>0</v>
+      </c>
+      <c r="P38" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17">
+      <c r="A39" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" t="s">
+        <v>59</v>
+      </c>
+      <c r="C39" t="s">
+        <v>60</v>
+      </c>
+      <c r="D39" t="s">
+        <v>63</v>
+      </c>
+      <c r="F39" t="s">
+        <v>69</v>
+      </c>
+      <c r="G39" t="s">
+        <v>92</v>
+      </c>
+      <c r="H39" t="s">
         <v>110</v>
-      </c>
-      <c r="L38">
-        <v>0</v>
-      </c>
-      <c r="M38">
-        <v>7</v>
-      </c>
-      <c r="N38" t="b">
-        <v>1</v>
-      </c>
-      <c r="O38" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15">
-      <c r="A39" t="s">
-        <v>52</v>
-      </c>
-      <c r="B39" t="s">
-        <v>57</v>
-      </c>
-      <c r="C39" t="s">
-        <v>58</v>
-      </c>
-      <c r="D39" t="s">
-        <v>61</v>
-      </c>
-      <c r="F39" t="s">
-        <v>67</v>
-      </c>
-      <c r="G39" t="s">
-        <v>90</v>
-      </c>
-      <c r="H39" t="s">
-        <v>108</v>
       </c>
       <c r="I39">
         <v>-8.382409832</v>
@@ -2504,42 +2738,48 @@
         <v>115.1953139</v>
       </c>
       <c r="K39" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L39">
         <v>1</v>
       </c>
       <c r="M39">
-        <v>2</v>
-      </c>
-      <c r="N39" t="b">
         <v>1</v>
       </c>
-      <c r="O39" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15">
+      <c r="N39">
+        <v>0</v>
+      </c>
+      <c r="O39">
+        <v>0</v>
+      </c>
+      <c r="P39" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17">
       <c r="A40" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B40" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C40" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D40" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F40" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H40" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I40">
         <v>-8.392661041</v>
@@ -2548,42 +2788,48 @@
         <v>115.1955531</v>
       </c>
       <c r="K40" t="s">
+        <v>112</v>
+      </c>
+      <c r="L40">
+        <v>0</v>
+      </c>
+      <c r="M40">
+        <v>0</v>
+      </c>
+      <c r="N40">
+        <v>0</v>
+      </c>
+      <c r="O40">
+        <v>0</v>
+      </c>
+      <c r="P40" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17">
+      <c r="A41" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" t="s">
+        <v>59</v>
+      </c>
+      <c r="C41" t="s">
+        <v>60</v>
+      </c>
+      <c r="D41" t="s">
+        <v>63</v>
+      </c>
+      <c r="F41" t="s">
+        <v>69</v>
+      </c>
+      <c r="G41" t="s">
+        <v>92</v>
+      </c>
+      <c r="H41" t="s">
         <v>110</v>
-      </c>
-      <c r="L40">
-        <v>0</v>
-      </c>
-      <c r="M40">
-        <v>8</v>
-      </c>
-      <c r="N40" t="b">
-        <v>1</v>
-      </c>
-      <c r="O40" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15">
-      <c r="A41" t="s">
-        <v>54</v>
-      </c>
-      <c r="B41" t="s">
-        <v>57</v>
-      </c>
-      <c r="C41" t="s">
-        <v>58</v>
-      </c>
-      <c r="D41" t="s">
-        <v>61</v>
-      </c>
-      <c r="F41" t="s">
-        <v>67</v>
-      </c>
-      <c r="G41" t="s">
-        <v>90</v>
-      </c>
-      <c r="H41" t="s">
-        <v>108</v>
       </c>
       <c r="I41">
         <v>-8.394319465000001</v>
@@ -2592,43 +2838,49 @@
         <v>115.1955146</v>
       </c>
       <c r="K41" t="s">
+        <v>112</v>
+      </c>
+      <c r="L41">
+        <v>0</v>
+      </c>
+      <c r="M41">
+        <v>0</v>
+      </c>
+      <c r="N41">
+        <v>0</v>
+      </c>
+      <c r="O41">
+        <v>0</v>
+      </c>
+      <c r="P41" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17">
+      <c r="A42" t="s">
+        <v>57</v>
+      </c>
+      <c r="B42" t="s">
+        <v>59</v>
+      </c>
+      <c r="C42" t="s">
+        <v>60</v>
+      </c>
+      <c r="D42" t="s">
+        <v>63</v>
+      </c>
+      <c r="F42" t="s">
+        <v>69</v>
+      </c>
+      <c r="G42" t="s">
+        <v>92</v>
+      </c>
+      <c r="H42" t="s">
         <v>110</v>
       </c>
-      <c r="L41">
-        <v>0</v>
-      </c>
-      <c r="M41">
-        <v>6</v>
-      </c>
-      <c r="N41" t="b">
-        <v>1</v>
-      </c>
-      <c r="O41" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15">
-      <c r="A42" t="s">
-        <v>55</v>
-      </c>
-      <c r="B42" t="s">
-        <v>57</v>
-      </c>
-      <c r="C42" t="s">
-        <v>58</v>
-      </c>
-      <c r="D42" t="s">
-        <v>61</v>
-      </c>
-      <c r="F42" t="s">
-        <v>67</v>
-      </c>
-      <c r="G42" t="s">
-        <v>90</v>
-      </c>
-      <c r="H42" t="s">
-        <v>108</v>
-      </c>
       <c r="I42">
         <v>0</v>
       </c>
@@ -2636,42 +2888,48 @@
         <v>0</v>
       </c>
       <c r="K42" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="L42">
         <v>3</v>
       </c>
       <c r="M42">
-        <v>8</v>
-      </c>
-      <c r="N42" t="b">
+        <v>2</v>
+      </c>
+      <c r="N42">
         <v>1</v>
       </c>
-      <c r="O42" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15">
+      <c r="O42">
+        <v>0</v>
+      </c>
+      <c r="P42" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17">
       <c r="A43" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B43" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C43" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D43" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F43" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G43" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H43" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I43">
         <v>-8.404993971</v>
@@ -2680,19 +2938,25 @@
         <v>115.1969283</v>
       </c>
       <c r="K43" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="L43">
         <v>0</v>
       </c>
       <c r="M43">
-        <v>2</v>
-      </c>
-      <c r="N43" t="b">
-        <v>1</v>
-      </c>
-      <c r="O43" t="s">
-        <v>112</v>
+        <v>0</v>
+      </c>
+      <c r="N43">
+        <v>0</v>
+      </c>
+      <c r="O43">
+        <v>0</v>
+      </c>
+      <c r="P43" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update INARA 2026-09-08 21:55:44
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -813,7 +813,7 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P2" t="b">
         <v>1</v>
@@ -863,7 +863,7 @@
         <v>0</v>
       </c>
       <c r="O3">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="P3" t="b">
         <v>1</v>
@@ -916,10 +916,10 @@
         <v>1</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="s">
         <v>114</v>
@@ -969,10 +969,10 @@
         <v>0</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q5" t="s">
         <v>114</v>
@@ -1022,10 +1022,10 @@
         <v>0</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6" t="s">
         <v>114</v>
@@ -1075,10 +1075,10 @@
         <v>0</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="s">
         <v>114</v>
@@ -1128,10 +1128,10 @@
         <v>0</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q8" t="s">
         <v>114</v>
@@ -1181,10 +1181,10 @@
         <v>0</v>
       </c>
       <c r="O9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9" t="s">
         <v>114</v>
@@ -1234,10 +1234,10 @@
         <v>0</v>
       </c>
       <c r="O10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q10" t="s">
         <v>114</v>
@@ -1287,10 +1287,10 @@
         <v>0</v>
       </c>
       <c r="O11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="s">
         <v>114</v>
@@ -1340,10 +1340,10 @@
         <v>0</v>
       </c>
       <c r="O12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q12" t="s">
         <v>114</v>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="O13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q13" t="s">
         <v>114</v>
@@ -1446,10 +1446,10 @@
         <v>0</v>
       </c>
       <c r="O14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q14" t="s">
         <v>114</v>
@@ -1499,10 +1499,10 @@
         <v>0</v>
       </c>
       <c r="O15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q15" t="s">
         <v>114</v>
@@ -1552,10 +1552,10 @@
         <v>0</v>
       </c>
       <c r="O16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q16" t="s">
         <v>114</v>
@@ -1605,10 +1605,10 @@
         <v>0</v>
       </c>
       <c r="O17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q17" t="s">
         <v>114</v>
@@ -1658,10 +1658,10 @@
         <v>0</v>
       </c>
       <c r="O18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q18" t="s">
         <v>114</v>
@@ -1711,10 +1711,10 @@
         <v>0</v>
       </c>
       <c r="O19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" t="s">
         <v>114</v>
@@ -1764,10 +1764,10 @@
         <v>0</v>
       </c>
       <c r="O20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q20" t="s">
         <v>114</v>
@@ -1817,10 +1817,10 @@
         <v>0</v>
       </c>
       <c r="O21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q21" t="s">
         <v>114</v>
@@ -1870,10 +1870,10 @@
         <v>0</v>
       </c>
       <c r="O22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q22" t="s">
         <v>114</v>
@@ -1923,10 +1923,10 @@
         <v>0</v>
       </c>
       <c r="O23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q23" t="s">
         <v>114</v>
@@ -1976,10 +1976,10 @@
         <v>0</v>
       </c>
       <c r="O24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q24" t="s">
         <v>114</v>
@@ -2029,10 +2029,10 @@
         <v>0</v>
       </c>
       <c r="O25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q25" t="s">
         <v>114</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="O26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q26" t="s">
         <v>114</v>
@@ -2135,10 +2135,10 @@
         <v>0</v>
       </c>
       <c r="O27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q27" t="s">
         <v>114</v>
@@ -2188,10 +2188,10 @@
         <v>1</v>
       </c>
       <c r="O28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q28" t="s">
         <v>114</v>
@@ -2241,10 +2241,10 @@
         <v>0</v>
       </c>
       <c r="O29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q29" t="s">
         <v>114</v>
@@ -2294,10 +2294,10 @@
         <v>0</v>
       </c>
       <c r="O30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q30" t="s">
         <v>114</v>
@@ -2347,10 +2347,10 @@
         <v>0</v>
       </c>
       <c r="O31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q31" t="s">
         <v>114</v>
@@ -2450,10 +2450,10 @@
         <v>0</v>
       </c>
       <c r="O33">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q33" t="s">
         <v>114</v>
@@ -2500,10 +2500,10 @@
         <v>0</v>
       </c>
       <c r="O34">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q34" t="s">
         <v>114</v>
@@ -2550,7 +2550,7 @@
         <v>1</v>
       </c>
       <c r="O35">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="P35" t="b">
         <v>1</v>
@@ -2600,10 +2600,10 @@
         <v>1</v>
       </c>
       <c r="O36">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q36" t="s">
         <v>114</v>
@@ -2650,10 +2650,10 @@
         <v>0</v>
       </c>
       <c r="O37">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q37" t="s">
         <v>114</v>
@@ -2700,10 +2700,10 @@
         <v>0</v>
       </c>
       <c r="O38">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="P38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q38" t="s">
         <v>114</v>
@@ -2750,10 +2750,10 @@
         <v>0</v>
       </c>
       <c r="O39">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q39" t="s">
         <v>114</v>
@@ -2800,10 +2800,10 @@
         <v>0</v>
       </c>
       <c r="O40">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q40" t="s">
         <v>114</v>
@@ -2850,10 +2850,10 @@
         <v>0</v>
       </c>
       <c r="O41">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q41" t="s">
         <v>114</v>
@@ -2900,10 +2900,10 @@
         <v>1</v>
       </c>
       <c r="O42">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q42" t="s">
         <v>114</v>
@@ -2950,10 +2950,10 @@
         <v>0</v>
       </c>
       <c r="O43">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q43" t="s">
         <v>114</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-09 08:17:24
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -813,10 +813,10 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="s">
         <v>114</v>
@@ -863,10 +863,10 @@
         <v>0</v>
       </c>
       <c r="O3">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="P3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q3" t="s">
         <v>114</v>
@@ -916,10 +916,10 @@
         <v>1</v>
       </c>
       <c r="O4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="s">
         <v>114</v>
@@ -969,10 +969,10 @@
         <v>0</v>
       </c>
       <c r="O5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="s">
         <v>114</v>
@@ -1022,10 +1022,10 @@
         <v>0</v>
       </c>
       <c r="O6">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="s">
         <v>114</v>
@@ -1075,10 +1075,10 @@
         <v>0</v>
       </c>
       <c r="O7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="s">
         <v>114</v>
@@ -1128,10 +1128,10 @@
         <v>0</v>
       </c>
       <c r="O8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="s">
         <v>114</v>
@@ -1181,10 +1181,10 @@
         <v>0</v>
       </c>
       <c r="O9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="s">
         <v>114</v>
@@ -1234,10 +1234,10 @@
         <v>0</v>
       </c>
       <c r="O10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="s">
         <v>114</v>
@@ -1287,10 +1287,10 @@
         <v>0</v>
       </c>
       <c r="O11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="s">
         <v>114</v>
@@ -1340,10 +1340,10 @@
         <v>0</v>
       </c>
       <c r="O12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="s">
         <v>114</v>
@@ -1393,10 +1393,10 @@
         <v>0</v>
       </c>
       <c r="O13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="s">
         <v>114</v>
@@ -2347,10 +2347,10 @@
         <v>0</v>
       </c>
       <c r="O31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q31" t="s">
         <v>114</v>
@@ -2400,10 +2400,10 @@
         <v>0</v>
       </c>
       <c r="O32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q32" t="s">
         <v>114</v>
@@ -2450,7 +2450,7 @@
         <v>0</v>
       </c>
       <c r="O33">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P33" t="b">
         <v>1</v>
@@ -2500,7 +2500,7 @@
         <v>0</v>
       </c>
       <c r="O34">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P34" t="b">
         <v>1</v>
@@ -2550,10 +2550,10 @@
         <v>1</v>
       </c>
       <c r="O35">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q35" t="s">
         <v>114</v>
@@ -2600,10 +2600,10 @@
         <v>1</v>
       </c>
       <c r="O36">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q36" t="s">
         <v>114</v>
@@ -2650,10 +2650,10 @@
         <v>0</v>
       </c>
       <c r="O37">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="P37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q37" t="s">
         <v>114</v>
@@ -2700,10 +2700,10 @@
         <v>0</v>
       </c>
       <c r="O38">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q38" t="s">
         <v>114</v>
@@ -2750,10 +2750,10 @@
         <v>0</v>
       </c>
       <c r="O39">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q39" t="s">
         <v>114</v>
@@ -2800,10 +2800,10 @@
         <v>0</v>
       </c>
       <c r="O40">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q40" t="s">
         <v>114</v>
@@ -2850,10 +2850,10 @@
         <v>0</v>
       </c>
       <c r="O41">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q41" t="s">
         <v>114</v>
@@ -2900,10 +2900,10 @@
         <v>1</v>
       </c>
       <c r="O42">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q42" t="s">
         <v>114</v>
@@ -2950,10 +2950,10 @@
         <v>0</v>
       </c>
       <c r="O43">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q43" t="s">
         <v>114</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-09 10:21:24
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -1446,10 +1446,10 @@
         <v>0</v>
       </c>
       <c r="O14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q14" t="s">
         <v>114</v>
@@ -1499,10 +1499,10 @@
         <v>0</v>
       </c>
       <c r="O15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q15" t="s">
         <v>114</v>
@@ -1552,10 +1552,10 @@
         <v>0</v>
       </c>
       <c r="O16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q16" t="s">
         <v>114</v>
@@ -1605,10 +1605,10 @@
         <v>0</v>
       </c>
       <c r="O17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="s">
         <v>114</v>
@@ -1658,10 +1658,10 @@
         <v>0</v>
       </c>
       <c r="O18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="s">
         <v>114</v>
@@ -1711,10 +1711,10 @@
         <v>0</v>
       </c>
       <c r="O19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q19" t="s">
         <v>114</v>
@@ -1764,10 +1764,10 @@
         <v>0</v>
       </c>
       <c r="O20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q20" t="s">
         <v>114</v>
@@ -1817,10 +1817,10 @@
         <v>0</v>
       </c>
       <c r="O21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q21" t="s">
         <v>114</v>
@@ -1870,10 +1870,10 @@
         <v>0</v>
       </c>
       <c r="O22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q22" t="s">
         <v>114</v>
@@ -1923,10 +1923,10 @@
         <v>0</v>
       </c>
       <c r="O23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q23" t="s">
         <v>114</v>
@@ -1976,10 +1976,10 @@
         <v>0</v>
       </c>
       <c r="O24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q24" t="s">
         <v>114</v>
@@ -2029,10 +2029,10 @@
         <v>0</v>
       </c>
       <c r="O25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q25" t="s">
         <v>114</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="O26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q26" t="s">
         <v>114</v>
@@ -2135,10 +2135,10 @@
         <v>0</v>
       </c>
       <c r="O27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q27" t="s">
         <v>114</v>
@@ -2188,10 +2188,10 @@
         <v>1</v>
       </c>
       <c r="O28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q28" t="s">
         <v>114</v>
@@ -2241,10 +2241,10 @@
         <v>0</v>
       </c>
       <c r="O29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q29" t="s">
         <v>114</v>
@@ -2294,10 +2294,10 @@
         <v>0</v>
       </c>
       <c r="O30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q30" t="s">
         <v>114</v>
@@ -2450,10 +2450,10 @@
         <v>0</v>
       </c>
       <c r="O33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q33" t="s">
         <v>114</v>
@@ -2500,10 +2500,10 @@
         <v>0</v>
       </c>
       <c r="O34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q34" t="s">
         <v>114</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-09 11:03:11
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -1234,10 +1234,10 @@
         <v>0</v>
       </c>
       <c r="O10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q10" t="s">
         <v>114</v>
@@ -1287,10 +1287,10 @@
         <v>0</v>
       </c>
       <c r="O11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="s">
         <v>114</v>
@@ -2450,10 +2450,10 @@
         <v>0</v>
       </c>
       <c r="O33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q33" t="s">
         <v>114</v>
@@ -2500,10 +2500,10 @@
         <v>0</v>
       </c>
       <c r="O34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q34" t="s">
         <v>114</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-09 12:04:36
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -813,10 +813,10 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="s">
         <v>114</v>
@@ -863,10 +863,10 @@
         <v>0</v>
       </c>
       <c r="O3">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="s">
         <v>114</v>
@@ -2400,10 +2400,10 @@
         <v>0</v>
       </c>
       <c r="O32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q32" t="s">
         <v>114</v>
@@ -2550,10 +2550,10 @@
         <v>1</v>
       </c>
       <c r="O35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q35" t="s">
         <v>114</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-11 10:19:10
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -813,7 +813,7 @@
         <v>1</v>
       </c>
       <c r="O2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="P2" t="b">
         <v>1</v>
@@ -863,7 +863,7 @@
         <v>0</v>
       </c>
       <c r="O3">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="P3" t="b">
         <v>1</v>
@@ -916,10 +916,10 @@
         <v>1</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="s">
         <v>114</v>
@@ -969,10 +969,10 @@
         <v>0</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q5" t="s">
         <v>114</v>
@@ -1022,10 +1022,10 @@
         <v>0</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6" t="s">
         <v>114</v>
@@ -1075,10 +1075,10 @@
         <v>0</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="s">
         <v>114</v>
@@ -1128,10 +1128,10 @@
         <v>0</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q8" t="s">
         <v>114</v>
@@ -1181,10 +1181,10 @@
         <v>0</v>
       </c>
       <c r="O9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9" t="s">
         <v>114</v>
@@ -1287,7 +1287,7 @@
         <v>0</v>
       </c>
       <c r="O11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P11" t="b">
         <v>1</v>
@@ -1340,10 +1340,10 @@
         <v>0</v>
       </c>
       <c r="O12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q12" t="s">
         <v>114</v>
@@ -1375,28 +1375,28 @@
         <v>100</v>
       </c>
       <c r="I13">
-        <v>-8.347617261</v>
+        <v>0</v>
       </c>
       <c r="J13">
-        <v>116.1690833</v>
+        <v>0</v>
       </c>
       <c r="K13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13">
         <v>0</v>
       </c>
       <c r="N13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q13" t="s">
         <v>114</v>
@@ -1446,10 +1446,10 @@
         <v>0</v>
       </c>
       <c r="O14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q14" t="s">
         <v>114</v>
@@ -1499,10 +1499,10 @@
         <v>0</v>
       </c>
       <c r="O15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q15" t="s">
         <v>114</v>
@@ -1817,10 +1817,10 @@
         <v>0</v>
       </c>
       <c r="O21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q21" t="s">
         <v>114</v>
@@ -1870,10 +1870,10 @@
         <v>0</v>
       </c>
       <c r="O22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q22" t="s">
         <v>114</v>
@@ -1923,10 +1923,10 @@
         <v>0</v>
       </c>
       <c r="O23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q23" t="s">
         <v>114</v>
@@ -2188,10 +2188,10 @@
         <v>1</v>
       </c>
       <c r="O28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q28" t="s">
         <v>114</v>
@@ -2241,10 +2241,10 @@
         <v>0</v>
       </c>
       <c r="O29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q29" t="s">
         <v>114</v>
@@ -2294,10 +2294,10 @@
         <v>0</v>
       </c>
       <c r="O30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q30" t="s">
         <v>114</v>
@@ -2450,7 +2450,7 @@
         <v>0</v>
       </c>
       <c r="O33">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="P33" t="b">
         <v>1</v>
@@ -2500,7 +2500,7 @@
         <v>0</v>
       </c>
       <c r="O34">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="P34" t="b">
         <v>1</v>
@@ -2650,10 +2650,10 @@
         <v>0</v>
       </c>
       <c r="O37">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q37" t="s">
         <v>114</v>
@@ -2700,10 +2700,10 @@
         <v>0</v>
       </c>
       <c r="O38">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q38" t="s">
         <v>114</v>
@@ -2750,10 +2750,10 @@
         <v>0</v>
       </c>
       <c r="O39">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q39" t="s">
         <v>114</v>
@@ -2800,10 +2800,10 @@
         <v>0</v>
       </c>
       <c r="O40">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q40" t="s">
         <v>114</v>
@@ -2832,28 +2832,28 @@
         <v>110</v>
       </c>
       <c r="I41">
-        <v>-8.394319465000001</v>
+        <v>0</v>
       </c>
       <c r="J41">
-        <v>115.1955146</v>
+        <v>0</v>
       </c>
       <c r="K41" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M41">
         <v>0</v>
       </c>
       <c r="N41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O41">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q41" t="s">
         <v>114</v>
@@ -2900,10 +2900,10 @@
         <v>1</v>
       </c>
       <c r="O42">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q42" t="s">
         <v>114</v>
@@ -2950,10 +2950,10 @@
         <v>0</v>
       </c>
       <c r="O43">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q43" t="s">
         <v>114</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-12 10:28:40
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -916,7 +916,7 @@
         <v>1</v>
       </c>
       <c r="O4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P4" t="b">
         <v>1</v>
@@ -969,7 +969,7 @@
         <v>0</v>
       </c>
       <c r="O5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P5" t="b">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         <v>0</v>
       </c>
       <c r="O6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P6" t="b">
         <v>1</v>
@@ -1075,7 +1075,7 @@
         <v>0</v>
       </c>
       <c r="O7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P7" t="b">
         <v>1</v>
@@ -1446,7 +1446,7 @@
         <v>0</v>
       </c>
       <c r="O14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P14" t="b">
         <v>1</v>
@@ -1499,7 +1499,7 @@
         <v>0</v>
       </c>
       <c r="O15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P15" t="b">
         <v>1</v>
@@ -1552,10 +1552,10 @@
         <v>0</v>
       </c>
       <c r="O16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q16" t="s">
         <v>114</v>
@@ -1711,10 +1711,10 @@
         <v>0</v>
       </c>
       <c r="O19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" t="s">
         <v>114</v>
@@ -1764,10 +1764,10 @@
         <v>0</v>
       </c>
       <c r="O20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q20" t="s">
         <v>114</v>
@@ -1923,7 +1923,7 @@
         <v>0</v>
       </c>
       <c r="O23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P23" t="b">
         <v>1</v>
@@ -2550,7 +2550,7 @@
         <v>1</v>
       </c>
       <c r="O35">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P35" t="b">
         <v>1</v>
@@ -2600,10 +2600,10 @@
         <v>1</v>
       </c>
       <c r="O36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q36" t="s">
         <v>114</v>

</xml_diff>